<commit_message>
Fix: 11 Bloomberg/NVIDIA rows were wrongly skipped; mark needs_manual for per-role verification
</commit_message>
<xml_diff>
--- a/applications_live.xlsx
+++ b/applications_live.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -449,6 +449,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,8 +471,6 @@
           <t>https://pru.wd5.myworkdayjobs.com/en-US/Careers/job/Newark-NJ-USA/Senior-Associate---Modeling--Remote-_R-119906</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -485,8 +488,6 @@
           <t>https://external-firstcitizens.icims.com/jobs/27452/job?mobile=false&amp;width=1140&amp;height=500&amp;bga=true&amp;needsRedirect=false&amp;jan1offset=-300&amp;jun1offset=-240</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -504,8 +505,6 @@
           <t>https://www.quadeye.com/careers/?gh_jid=7956444002</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -523,10 +522,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Index-Quant-Researcher-New-York/12019</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -546,10 +549,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Senior-Quantitative-Analyst-Home-Price-Modeling-EXT/13448</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -569,8 +576,6 @@
           <t>https://jobs.ashbyhq.com/ramp/d204e136-2749-42de-82b4-88a0dd352090</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -588,10 +593,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Index-Quant-Researcher-London/12022</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -611,8 +620,6 @@
           <t>https://www.uber.com/global/en/careers/list/144266/</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -630,8 +637,6 @@
           <t>https://jobs.lever.co/voleon/ce0bda1f-3d5a-44ac-8ab3-8578d49d344c</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -649,8 +654,6 @@
           <t>https://www.uber.com/global/en/careers/list/137616/?uclick_id=3d50b1bf-893e-47f6-ab28-595a9c2921fb</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -668,8 +671,6 @@
           <t>https://search.jobs.barclays/job/-/-/13015/85253243872?src=JB-12860</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -687,8 +688,6 @@
           <t>https://career.mlp.com/careers/job/755938464555?domain=mlp.com&amp;utm_source=linkedin</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -706,8 +705,6 @@
           <t>https://www.capitalonecareers.com/job/mclean/senior-associate-data-scientist-applied-ai/1732/85271909856</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -725,10 +722,14 @@
           <t>https://bloomberg.avature.net/careers/Private?jobId=13613</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -748,10 +749,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Senior-Language-Modeling-Research-Engineer-Artificial-Intelligence/4373</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -771,10 +776,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Senior-Quant-Analyst-Trading-Decision-Tools-Equities/16017</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -794,10 +803,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Senior-Machine-Learning-Engineer-BLAW-BGOV-BTAX/16695</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -817,8 +830,6 @@
           <t>https://explore.jobs.netflix.net/careers/job/790315191475-machine-learning-scientist-5-production-science-usa-remote?domain=netflix.com&amp;microsite=netflix.com</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -836,8 +847,6 @@
           <t>https://jobs.louisvuitton.com/en/search-page/job/senior-data-scientist-analytics-and-ai-data-united-states-new-york-LVM32143?sType=Linkedin</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -855,10 +864,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Bloomberg-Product-Oversight-Data-Scientist/18817</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -878,10 +891,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Bloomberg-Intelligence-Technology-Equity-Research-Analyst-Cybersecurity/17395</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -901,10 +918,14 @@
           <t>https://nvidia.wd5.myworkdayjobs.com/NVIDIAExternalCareerSite/job/US-CA-Santa-Clara/Senior-Deep-Learning-Scientist--Multimodal-Agentic-RL_JR2022039</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -924,10 +945,14 @@
           <t>https://bloomberg.avature.net/careers/JobDetail/Bloomberg-Intelligence-Credit-Research-Analyst-US-Auto-Suppliers-Retailers/20740</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>skipped_already_applied</t>
+          <t>needs_manual</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Existing account/record found, but no evidence this specific role was applied to - verify before applying</t>
         </is>
       </c>
     </row>
@@ -947,8 +972,6 @@
           <t>https://abglobal.wd1.myworkdayjobs.com/alliancebernsteincareers/job/New-York-New-York/Quantitative-Researcher_R0019166-1</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -966,8 +989,6 @@
           <t>https://careers.bankofamerica.com/en-us/job-detail/26003477/vp-genai-quant-developer-new-york-new-york-united-states-esomprank-mauoyxvskp-8</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -985,8 +1006,6 @@
           <t>https://jobs.ashbyhq.com/openai/90c711dc-5f50-46e3-a5ab-82359a56d683/application</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1004,8 +1023,6 @@
           <t>https://careers.moodys.com/en/job/-/-/49841/98147683616?utm_source=linkedin&amp;jobPipeline=LinkedIn</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1023,8 +1040,6 @@
           <t>https://jobs.apple.com/en-us/details/200661360-3337/senior-applied-scientist-multilingual-ai-evaluation</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1042,8 +1057,6 @@
           <t>https://block.xyz/careers/jobs/5412922008</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>